<commit_message>
fixed O2 mapping and some minor visuals fixes
</commit_message>
<xml_diff>
--- a/data/C19RM mapping.xlsx
+++ b/data/C19RM mapping.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tommeijer/Git/RSSH-Budget-PF-Dashboard/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tommeijer/POC/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{376815B3-F551-AB43-ADB1-EF8FE68DB060}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A81DA1D-601D-1744-BFDD-11C9203E7EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="42">
   <si>
     <t>RSSH/PP: Laboratory systems (including national and peripheral)</t>
   </si>
@@ -153,13 +153,19 @@
   </si>
   <si>
     <t>Case management, clinical operations, and therapeutics - Case management</t>
+  </si>
+  <si>
+    <t>Case management, clinical operations and therapeutics (excl O2)</t>
+  </si>
+  <si>
+    <t>Case management, clinical operations and therapeutics (O2 only)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -169,6 +175,12 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -195,9 +207,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="64" bestFit="1" customWidth="1"/>
@@ -548,16 +561,16 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>8</v>
+      <c r="A2" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>33</v>
+      <c r="A3" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
@@ -565,7 +578,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
         <v>34</v>
@@ -573,7 +586,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
@@ -581,55 +594,55 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>1</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>1</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s">
         <v>1</v>
@@ -637,7 +650,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
         <v>1</v>
@@ -645,7 +658,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B14" t="s">
         <v>1</v>
@@ -653,31 +666,31 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>35</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>2</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="B18" t="s">
         <v>2</v>
@@ -685,31 +698,31 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B19" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="B20" t="s">
-        <v>34</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B22" t="s">
         <v>34</v>
@@ -717,7 +730,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="B23" t="s">
         <v>34</v>
@@ -725,7 +738,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B24" t="s">
         <v>34</v>
@@ -733,7 +746,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B25" t="s">
         <v>34</v>
@@ -741,23 +754,23 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B26" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B28" t="s">
         <v>4</v>
@@ -765,23 +778,39 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B29" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>21</v>
+      </c>
+      <c r="B31" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>22</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B32" t="s">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A1863">
-    <sortCondition ref="A2:A1863"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:A1865">
+    <sortCondition ref="A4:A1865"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>